<commit_message>
Correct postal code to 10123 in price list and spreadsheet
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cjenik-chokai.xlsx
+++ b/cjenik-chokai.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="4"/>
+  <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Cjenik" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
   <authors>
     <author>CHOKAI</author>
   </authors>
@@ -41,6 +41,27 @@
 Kod buduće promjene cijene ovaj stupac zadržava cijenu s referentnog datuma; mijenja se samo stupac C.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>8</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>59</xdr:colOff>
+                <xdr:row>6</xdr:row>
+                <xdr:rowOff>12</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
   </commentList>
 </comments>
@@ -55,7 +76,7 @@
     <t xml:space="preserve">CHOKAI, obrt za računalne i poslovne usluge, vl. Matko Stanković</t>
   </si>
   <si>
-    <t xml:space="preserve">Petrova 84, 10000 Zagreb, Hrvatska</t>
+    <t xml:space="preserve">Petrova 84, 10123 Zagreb, Hrvatska</t>
   </si>
   <si>
     <t xml:space="preserve">OIB: 64389569095    MBO: 98086448    Obrtnica: 21010143794</t>

</xml_diff>